<commit_message>
Cedar Chic só em decant (promoção de/por) + suporte a 'só decant' e preço riscado
</commit_message>
<xml_diff>
--- a/modelos/Maison-Galbano-Catalogo.xlsx
+++ b/modelos/Maison-Galbano-Catalogo.xlsx
@@ -654,7 +654,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R300"/>
+  <dimension ref="A1:S300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -675,6 +675,7 @@
     <col width="10" customWidth="1" min="16" max="16"/>
     <col width="18" customWidth="1" min="17" max="17"/>
     <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="16" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -768,6 +769,11 @@
           <t>preco_decant</t>
         </is>
       </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>preco_decant_de</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="57" t="inlineStr">
@@ -11886,23 +11892,93 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="4" t="n"/>
-      <c r="B136" s="4" t="n"/>
-      <c r="C136" s="4" t="n"/>
-      <c r="D136" s="4" t="n"/>
-      <c r="E136" s="4" t="n"/>
-      <c r="F136" s="4" t="n"/>
-      <c r="G136" s="4" t="n"/>
-      <c r="H136" s="4" t="n"/>
-      <c r="I136" s="4" t="n"/>
-      <c r="J136" s="4" t="n"/>
-      <c r="K136" s="4" t="n"/>
-      <c r="L136" s="4" t="n"/>
-      <c r="M136" s="4" t="n"/>
-      <c r="N136" s="4" t="n"/>
-      <c r="O136" s="4" t="n"/>
-      <c r="P136" s="4" t="n"/>
-      <c r="Q136" s="4" t="n"/>
+      <c r="A136" s="4" t="inlineStr">
+        <is>
+          <t>MG135</t>
+        </is>
+      </c>
+      <c r="B136" s="4" t="inlineStr">
+        <is>
+          <t>Carolina Herrera</t>
+        </is>
+      </c>
+      <c r="C136" s="4" t="inlineStr">
+        <is>
+          <t>Cedar Chic</t>
+        </is>
+      </c>
+      <c r="D136" s="4" t="inlineStr">
+        <is>
+          <t>Eau de Parfum</t>
+        </is>
+      </c>
+      <c r="E136" s="4" t="inlineStr">
+        <is>
+          <t>100 ml</t>
+        </is>
+      </c>
+      <c r="F136" s="4" t="inlineStr">
+        <is>
+          <t>Nicho</t>
+        </is>
+      </c>
+      <c r="G136" s="4" t="inlineStr">
+        <is>
+          <t>Compartilhável</t>
+        </is>
+      </c>
+      <c r="H136" s="4" t="inlineStr">
+        <is>
+          <t>Amadeirado floral aldeídico</t>
+        </is>
+      </c>
+      <c r="I136" s="4" t="inlineStr">
+        <is>
+          <t>Acorde limpo, bergamota</t>
+        </is>
+      </c>
+      <c r="J136" s="4" t="inlineStr">
+        <is>
+          <t>Flor de laranjeira</t>
+        </is>
+      </c>
+      <c r="K136" s="4" t="inlineStr">
+        <is>
+          <t>Trio de cedros, almíscar branco</t>
+        </is>
+      </c>
+      <c r="L136" s="4" t="inlineStr">
+        <is>
+          <t>Dia a dia</t>
+        </is>
+      </c>
+      <c r="M136" s="4" t="inlineStr">
+        <is>
+          <t>Da Confidential Collection, a linha mais exclusiva de Carolina Herrera. Abre limpo e luminoso, com um acorde de frescor e bergamota. No coração, a flor de laranjeira traz uma elegância delicada. O fundo de um trio de cedros com almíscar branco deixa um rastro amadeirado, sofisticado e aconchegante. Compartilhável.</t>
+        </is>
+      </c>
+      <c r="N136" s="4" t="inlineStr"/>
+      <c r="O136" s="4" t="inlineStr">
+        <is>
+          <t>só decant</t>
+        </is>
+      </c>
+      <c r="P136" s="4" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="Q136" s="4" t="inlineStr"/>
+      <c r="R136" t="inlineStr">
+        <is>
+          <t>199,99</t>
+        </is>
+      </c>
+      <c r="S136" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="4" t="n"/>
@@ -15046,7 +15122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -15198,7 +15274,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>sim ou não. "não" mostra "Sob consulta"</t>
+          <t>sim ou não. "não" mostra "Sob consulta" Use "só decant" quando você vende só o decant: o frasco não aparece no site.</t>
         </is>
       </c>
     </row>
@@ -15239,10 +15315,22 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr"/>
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>preco_decant_de</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Opcional. Preço "de" do decant numa promoção (aparece riscado). Ex.: 240,00 com preco_decant 199,99.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="A19" s="6" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>Depois de salvar, o site atualiza sozinho em até 1 hora.</t>
         </is>

</xml_diff>

<commit_message>
Foto: Armaf Club de Nuit Woman (MG136)
</commit_message>
<xml_diff>
--- a/modelos/Maison-Galbano-Catalogo.xlsx
+++ b/modelos/Maison-Galbano-Catalogo.xlsx
@@ -11981,23 +11981,89 @@
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="4" t="n"/>
-      <c r="B137" s="4" t="n"/>
-      <c r="C137" s="4" t="n"/>
-      <c r="D137" s="4" t="n"/>
-      <c r="E137" s="4" t="n"/>
-      <c r="F137" s="4" t="n"/>
-      <c r="G137" s="4" t="n"/>
-      <c r="H137" s="4" t="n"/>
-      <c r="I137" s="4" t="n"/>
-      <c r="J137" s="4" t="n"/>
-      <c r="K137" s="4" t="n"/>
-      <c r="L137" s="4" t="n"/>
-      <c r="M137" s="4" t="n"/>
-      <c r="N137" s="4" t="n"/>
-      <c r="O137" s="4" t="n"/>
-      <c r="P137" s="4" t="n"/>
-      <c r="Q137" s="4" t="n"/>
+      <c r="A137" s="4" t="inlineStr">
+        <is>
+          <t>MG136</t>
+        </is>
+      </c>
+      <c r="B137" s="4" t="inlineStr">
+        <is>
+          <t>Armaf</t>
+        </is>
+      </c>
+      <c r="C137" s="4" t="inlineStr">
+        <is>
+          <t>Club de Nuit Woman</t>
+        </is>
+      </c>
+      <c r="D137" s="4" t="inlineStr">
+        <is>
+          <t>Eau de Parfum</t>
+        </is>
+      </c>
+      <c r="E137" s="4" t="inlineStr">
+        <is>
+          <t>105 ml</t>
+        </is>
+      </c>
+      <c r="F137" s="4" t="inlineStr">
+        <is>
+          <t>Árabe</t>
+        </is>
+      </c>
+      <c r="G137" s="4" t="inlineStr">
+        <is>
+          <t>Feminino</t>
+        </is>
+      </c>
+      <c r="H137" s="4" t="inlineStr">
+        <is>
+          <t>Floral frutado chypre</t>
+        </is>
+      </c>
+      <c r="I137" s="4" t="inlineStr">
+        <is>
+          <t>Laranja, bergamota, toranja, pêssego</t>
+        </is>
+      </c>
+      <c r="J137" s="4" t="inlineStr">
+        <is>
+          <t>Rosa, jasmim, gerânio, lichia</t>
+        </is>
+      </c>
+      <c r="K137" s="4" t="inlineStr">
+        <is>
+          <t>Patchouli, baunilha, almíscar, vetiver</t>
+        </is>
+      </c>
+      <c r="L137" s="4" t="inlineStr">
+        <is>
+          <t>Dia a dia, Assinatura</t>
+        </is>
+      </c>
+      <c r="M137" s="4" t="inlineStr">
+        <is>
+          <t>Uma joia da Armaf para a mulher elegante. Abre luminoso e suculento, com laranja, bergamota, toranja e pêssego. No coração, rosa, jasmim, gerânio e lichia formam um buquê sofisticado. O fundo de patchouli, baunilha, almíscar e vetiver deixa um rastro chique e marcante, uma assinatura de luxo para o dia a dia. Feminino.</t>
+        </is>
+      </c>
+      <c r="N137" s="4" t="inlineStr">
+        <is>
+          <t>350,00</t>
+        </is>
+      </c>
+      <c r="O137" s="4" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="P137" s="4" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="Q137" s="4" t="inlineStr"/>
+      <c r="R137" t="inlineStr"/>
+      <c r="S137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="4" t="n"/>

</xml_diff>